<commit_message>
chore: standardize render output to video/output + gitignore media/env
- stage-planned-images.ts + list-image-prompts.ts now resolve video/output/<slug>
  (matches the /create-video SKILL; pipeline already follows the script.json dir).
- Migrated all existing renders into video/output/; queue.xlsx result paths updated.
- .gitignore: keep the repo code-only — exclude generated/source media
  (video/output, podcast/output, podcast/_runs, video|podcast input images/
  footage/voice, scratch mockup media) and env. Anchored /SFX/ to root so the
  tracked assets/sfx SFX library is NOT dropped on case-insensitive filesystems.
- Untracked existing media from the index (files kept on disk).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video/input/queue.xlsx
+++ b/video/input/queue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="96">
   <si>
     <t>source</t>
   </si>
@@ -82,7 +82,7 @@
     <t>79 players Part 1</t>
   </si>
   <si>
-    <t>output/79-bom-tan-chuyen-nhuong-he-p1/video.mp4</t>
+    <t>video/output/79-bom-tan-chuyen-nhuong-he-p1/video.mp4</t>
   </si>
   <si>
     <t>video/input/79-bom-tan-chuyen-nhuong-he-p2/79-bom-tan-chuyen-nhuong-he-p2.txt</t>
@@ -94,7 +94,7 @@
     <t>79 players Part 2</t>
   </si>
   <si>
-    <t>output/79-bom-tan-chuyen-nhuong-he-p2/video.mp4</t>
+    <t>video/output/79-bom-tan-chuyen-nhuong-he-p2/video.mp4</t>
   </si>
   <si>
     <t>video/input/79-bom-tan-chuyen-nhuong-he-p3/79-bom-tan-chuyen-nhuong-he-p3.txt</t>
@@ -106,7 +106,7 @@
     <t>79 players Part 3</t>
   </si>
   <si>
-    <t>output/79-bom-tan-chuyen-nhuong-he-p3/video.mp4</t>
+    <t>video/output/79-bom-tan-chuyen-nhuong-he-p3/video.mp4</t>
   </si>
   <si>
     <t>video/input/79-bom-tan-chuyen-nhuong-he-p4/79-bom-tan-chuyen-nhuong-he-p4.txt</t>
@@ -118,7 +118,7 @@
     <t>79 players Part 4</t>
   </si>
   <si>
-    <t>output/79-bom-tan-chuyen-nhuong-he-p4/video.mp4</t>
+    <t>video/output/79-bom-tan-chuyen-nhuong-he-p4/video.mp4</t>
   </si>
   <si>
     <t>video/input/79-bom-tan-chuyen-nhuong-he-p5/79-bom-tan-chuyen-nhuong-he-p5.txt</t>
@@ -130,103 +130,103 @@
     <t>79 players Part 5</t>
   </si>
   <si>
-    <t>output/79-bom-tan-chuyen-nhuong-he-p5/video.mp4</t>
+    <t>video/output/79-bom-tan-chuyen-nhuong-he-p5/video.mp4</t>
   </si>
   <si>
     <t>video/input/argentina-worldcup/argentina-worldcup.txt</t>
   </si>
   <si>
-    <t>output/argentina-worldcup/video.mp4</t>
+    <t>video/output/argentina-worldcup/video.mp4</t>
   </si>
   <si>
     <t>video/input/portugal-worldcup/portugal-worldcup.txt</t>
   </si>
   <si>
-    <t>output/portugal-worldcup/video.mp4</t>
+    <t>video/output/portugal-worldcup/video.mp4</t>
   </si>
   <si>
     <t>video/input/nxgn-2026-teenage-sensations/nxgn-2026-teenage-sensations.txt</t>
   </si>
   <si>
-    <t>output/nxgn-2026-teenage-sensations/video.mp4</t>
+    <t>video/output/nxgn-2026-teenage-sensations/video.mp4</t>
   </si>
   <si>
     <t>video/input/sao-lon-bo-lo-world-cup-2026/sao-lon-bo-lo-world-cup-2026.txt</t>
   </si>
   <si>
-    <t>output/sao-lon-bo-lo-world-cup-2026/video.mp4</t>
+    <t>video/output/sao-lon-bo-lo-world-cup-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/haaland-ra-mat-world-cup-2026/haaland-ra-mat-world-cup-2026.txt</t>
   </si>
   <si>
-    <t>output/haaland-ra-mat-world-cup-2026/video.mp4</t>
+    <t>video/output/haaland-ra-mat-world-cup-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/ung-vien-chiec-giay-vang-world-cup-2026/ung-vien-chiec-giay-vang-world-cup-2026.txt</t>
   </si>
   <si>
-    <t>output/ung-vien-chiec-giay-vang-world-cup-2026/video.mp4</t>
+    <t>video/output/ung-vien-chiec-giay-vang-world-cup-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/mexico-vs-nam-phi-khai-mac-world-cup-2026/mexico-vs-nam-phi-khai-mac-world-cup-2026.txt</t>
   </si>
   <si>
-    <t>output/mexico-vs-nam-phi-khai-mac-world-cup-2026/video.mp4</t>
+    <t>video/output/mexico-vs-nam-phi-khai-mac-world-cup-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/harry-kane-dua-qua-bong-vang-2026/harry-kane-dua-qua-bong-vang-2026.txt</t>
   </si>
   <si>
-    <t>output/harry-kane-dua-qua-bong-vang-2026/video.mp4</t>
+    <t>video/output/harry-kane-dua-qua-bong-vang-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/nhan-dinh-my-vs-paraguay-wc-2026/nhan-dinh-my-vs-paraguay-wc-2026.txt</t>
   </si>
   <si>
-    <t>output/nhan-dinh-my-vs-paraguay-wc-2026/video.mp4</t>
+    <t>video/output/nhan-dinh-my-vs-paraguay-wc-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/nhan-dinh-han-quoc-vs-sec-wc-2026/nhan-dinh-han-quoc-vs-sec-wc-2026.txt</t>
   </si>
   <si>
-    <t>output/nhan-dinh-han-quoc-vs-sec-wc-2026/video.mp4</t>
+    <t>video/output/nhan-dinh-han-quoc-vs-sec-wc-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/nhan-dinh-canada-vs-bosnia-wc-2026/nhan-dinh-canada-vs-bosnia-wc-2026.txt</t>
   </si>
   <si>
-    <t>output/nhan-dinh-canada-vs-bosnia-wc-2026/video.mp4</t>
+    <t>video/output/nhan-dinh-canada-vs-bosnia-wc-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/hop-bao-thomas-tuchel-tuyen-anh-wc-2026/hop-bao-thomas-tuchel-tuyen-anh-wc-2026.txt</t>
   </si>
   <si>
-    <t>output/hop-bao-thomas-tuchel-tuyen-anh-wc-2026/video.mp4</t>
+    <t>video/output/hop-bao-thomas-tuchel-tuyen-anh-wc-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/garnachofunny/garnachofunny.txt</t>
   </si>
   <si>
-    <t>output/garnachofunny/video.mp4</t>
+    <t>video/output/garnachofunny/video.mp4</t>
   </si>
   <si>
     <t>video/input/diogo-dalot-ronaldo-va-diogo-jota/diogo-dalot-ronaldo-va-diogo-jota.txt</t>
   </si>
   <si>
-    <t>output/diogo-dalot-ronaldo-va-diogo-jota/video.mp4</t>
+    <t>video/output/diogo-dalot-ronaldo-va-diogo-jota/video.mp4</t>
   </si>
   <si>
     <t>video/input/tuyen-phap-thua-bo-bien-nga-chieu-sau-doi-hinh/tuyen-phap-thua-bo-bien-nga-chieu-sau-doi-hinh.txt</t>
   </si>
   <si>
-    <t>output/tuyen-phap-thua-bo-bien-nga-chieu-sau-doi-hinh/video.mp4</t>
+    <t>video/output/tuyen-phap-thua-bo-bien-nga-chieu-sau-doi-hinh/video.mp4</t>
   </si>
   <si>
     <t>video/input/ancelotti-va-brazil-giac-mo-world-cup/ancelotti-va-brazil-giac-mo-world-cup.txt</t>
   </si>
   <si>
-    <t>output/ancelotti-va-brazil-giac-mo-world-cup/video.mp4</t>
+    <t>video/output/ancelotti-va-brazil-giac-mo-world-cup/video.mp4</t>
   </si>
   <si>
     <t>video/input/mbappe-ronaldo-messi-doi-lap/mbappe-ronaldo-messi-doi-lap.txt</t>
@@ -235,7 +235,7 @@
     <t>Mbappe: Ronaldo và Messi đối lập ở mọi khía cạnh</t>
   </si>
   <si>
-    <t>output/mbappe-ronaldo-messi-doi-lap/video.mp4</t>
+    <t>video/output/mbappe-ronaldo-messi-doi-lap/video.mp4</t>
   </si>
   <si>
     <t>video/input/portugal-chile-ratings/portugal-chile-ratings.txt</t>
@@ -244,7 +244,7 @@
     <t>Chấm điểm Bồ Đào Nha 2-1 Chile: Bruno Fernandes rực sáng</t>
   </si>
   <si>
-    <t>output/portugal-chile-ratings/video.mp4</t>
+    <t>video/output/portugal-chile-ratings/video.mp4</t>
   </si>
   <si>
     <t>video/input/fifa-luat-hat-quoc-ca-moi/fifa-luat-hat-quoc-ca-moi.txt</t>
@@ -253,7 +253,7 @@
     <t>FIFA thay đổi nghi lễ hát quốc ca tại World Cup 2026</t>
   </si>
   <si>
-    <t>output/fifa-luat-hat-quoc-ca-moi/video.mp4</t>
+    <t>video/output/fifa-luat-hat-quoc-ca-moi/video.mp4</t>
   </si>
   <si>
     <t>video/input/england-new-zealand-ratings/england-new-zealand-ratings.txt</t>
@@ -262,7 +262,7 @@
     <t>Chấm điểm tuyển Anh vs New Zealand: Harry Kane tỏa sáng</t>
   </si>
   <si>
-    <t>output/england-new-zealand-ratings/video.mp4</t>
+    <t>video/output/england-new-zealand-ratings/video.mp4</t>
   </si>
   <si>
     <t>video/input/world-cup-2026-last-dance/world-cup-2026-last-dance.txt</t>
@@ -271,25 +271,37 @@
     <t>8 siêu sao và vũ điệu cuối cùng tại World Cup 2026</t>
   </si>
   <si>
-    <t>output/world-cup-2026-last-dance/video.mp4</t>
+    <t>video/output/world-cup-2026-last-dance/video.mp4</t>
   </si>
   <si>
     <t>video/input/mbappe-world-cup-cuu-canh-sau-mua-de-quen/mbappe-world-cup-cuu-canh-sau-mua-de-quen.txt</t>
   </si>
   <si>
-    <t>planned</t>
+    <t>video/output/mbappe-world-cup-cuu-canh-sau-mua-de-quen/video.mp4</t>
   </si>
   <si>
     <t>video/input/tam-cap-anh-em-ruot-tai-world-cup-2026/tam-cap-anh-em-ruot-tai-world-cup-2026.txt</t>
   </si>
   <si>
+    <t>video/output/tam-cap-anh-em-ruot-tai-world-cup-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/sau-cuoc-tranh-cai-chon-nguoi-wc-2026/sau-cuoc-tranh-cai-chon-nguoi-wc-2026.txt</t>
   </si>
   <si>
+    <t>video/output/sau-cuoc-tranh-cai-chon-nguoi-wc-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/eriksen-tinh-tao-sau-khi-nga-quy/eriksen-tinh-tao-sau-khi-nga-quy.txt</t>
   </si>
   <si>
+    <t>video/output/eriksen-tinh-tao-sau-khi-nga-quy/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/mourinho-tro-lai-real-madrid/mourinho-tro-lai-real-madrid.txt</t>
+  </si>
+  <si>
+    <t>video/output/mourinho-tro-lai-real-madrid/video.mp4</t>
   </si>
 </sst>
 </file>
@@ -1132,44 +1144,59 @@
         <v>85</v>
       </c>
     </row>
-    <row r="30" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>86</v>
       </c>
       <c r="E30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="31" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>88</v>
       </c>
       <c r="E31" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="32" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="33" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F32" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E33" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="34" ht="14.4" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F33" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="34" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E34" t="s">
-        <v>87</v>
+        <v>11</v>
+      </c>
+      <c r="F34" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content: mark WC2026 MD2 previews done in queue (rows 69-72)
Spain-Saudi, Belgium-Iran, Uruguay-Cabo Verde, NZ-Egypt previews rendered.
mp4 outputs live under gitignored video/output.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video/input/queue.xlsx
+++ b/video/input/queue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="183">
   <si>
     <t>source</t>
   </si>
@@ -541,7 +541,7 @@
     <t>match-preview WC2026 bang H MD2</t>
   </si>
   <si>
-    <t>planned</t>
+    <t>video/output/nhan-dinh-tay-ban-nha-vs-saudi-arabia-wc-2026/video.mp4</t>
   </si>
   <si>
     <t>video/input/nhan-dinh-bi-vs-iran-wc-2026/nhan-dinh-bi-vs-iran-wc-2026.txt</t>
@@ -550,10 +550,19 @@
     <t>match-preview WC2026 bang G MD2</t>
   </si>
   <si>
+    <t>video/output/nhan-dinh-bi-vs-iran-wc-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/nhan-dinh-uruguay-vs-cabo-verde-wc-2026/nhan-dinh-uruguay-vs-cabo-verde-wc-2026.txt</t>
   </si>
   <si>
+    <t>video/output/nhan-dinh-uruguay-vs-cabo-verde-wc-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/nhan-dinh-new-zealand-vs-ai-cap-wc-2026/nhan-dinh-new-zealand-vs-ai-cap-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-new-zealand-vs-ai-cap-wc-2026/video.mp4</t>
   </si>
 </sst>
 </file>
@@ -2024,7 +2033,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>173</v>
       </c>
@@ -2032,10 +2041,13 @@
         <v>174</v>
       </c>
       <c r="E69" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>176</v>
       </c>
@@ -2043,29 +2055,38 @@
         <v>177</v>
       </c>
       <c r="E70" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="F70" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D71" t="s">
         <v>174</v>
       </c>
       <c r="E71" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="F71" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D72" t="s">
         <v>177</v>
       </c>
       <c r="E72" t="s">
-        <v>175</v>
+        <v>9</v>
+      </c>
+      <c r="F72" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content: add WC2026 preview/recap batches + new podcast stories
video/input: new WC2026 nhan-dinh (match previews) and cham-diem (player
ratings) batches plus assorted single pieces, each with .txt + images-plan.json
(+ anh-can-tao.md / grok-prompts.md where present); refresh existing
nhan-dinh + mexico-vs-nam-phi sources and video queue.xlsx.

podcast: add story71-79 scripts and update podcast queue.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video/input/queue.xlsx
+++ b/video/input/queue.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79AD54A-B77C-4779-809A-1D211D253062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="queue" state="visible" r:id="rId4"/>
+    <sheet name="queue" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="214">
   <si>
     <t>source</t>
   </si>
@@ -563,19 +569,112 @@
   </si>
   <si>
     <t>video/output/nhan-dinh-new-zealand-vs-ai-cap-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-duc-vs-bo-bien-nga-wc-2026/cham-diem-duc-vs-bo-bien-nga-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/cham-diem-duc-vs-bo-bien-nga-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-ha-lan-vs-thuy-dien-wc-2026/cham-diem-ha-lan-vs-thuy-dien-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/cham-diem-ha-lan-vs-thuy-dien-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/3-ky-luc-cho-messi-o-tran-gap-ao/3-ky-luc-cho-messi-o-tran-gap-ao.txt</t>
+  </si>
+  <si>
+    <t>video/output/3-ky-luc-cho-messi-o-tran-gap-ao/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/yamal-messi-ro-rang-gioi-nhat-lich-su/yamal-messi-ro-rang-gioi-nhat-lich-su.txt</t>
+  </si>
+  <si>
+    <t>video/output/yamal-messi-ro-rang-gioi-nhat-lich-su/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/henry-doi-giong-ve-cristiano-ronaldo/henry-doi-giong-ve-cristiano-ronaldo.txt</t>
+  </si>
+  <si>
+    <t>video/output/henry-doi-giong-ve-cristiano-ronaldo/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-argentina-vs-ao-wc-2026/nhan-dinh-argentina-vs-ao-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-argentina-vs-ao-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-phap-vs-iraq-wc-2026/nhan-dinh-phap-vs-iraq-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>match-preview</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-phap-vs-iraq-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-na-uy-vs-senegal-wc-2026/nhan-dinh-na-uy-vs-senegal-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-na-uy-vs-senegal-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-jordan-vs-algeria-wc-2026/nhan-dinh-jordan-vs-algeria-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-jordan-vs-algeria-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-bi-vs-iran-lukaku-mo-nhat/cham-diem-bi-vs-iran-lukaku-mo-nhat.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite</t>
+  </si>
+  <si>
+    <t>Render failed</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-tay-ban-nha-vs-arab-saudi-oyarzabal/cham-diem-tay-ban-nha-vs-arab-saudi-oyarzabal.txt</t>
+  </si>
+  <si>
+    <t>video/input/owen-bao-ve-ronaldo-sau-tran-hoa-chdc-congo/owen-bao-ve-ronaldo-sau-tran-hoa-chdc-congo.txt</t>
+  </si>
+  <si>
+    <t>video/input/conceicao-bo-dao-nha-khong-co-nghia-vu-chuyen-cho-ronaldo/conceicao-bo-dao-nha-khong-co-nghia-vu-chuyen-cho-ronaldo.txt</t>
+  </si>
+  <si>
+    <t>video/input/top-10-cau-thu-vi-dai-nhat-lich-su-world-cup/top-10-cau-thu-vi-dai-nhat-lich-su-world-cup.txt</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-bo-dao-nha-vs-uzbekistan-wc-2026/nhan-dinh-bo-dao-nha-vs-uzbekistan-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-bo-dao-nha-vs-uzbekistan-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-anh-vs-ghana-wc-2026/nhan-dinh-anh-vs-ghana-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-panama-vs-croatia-wc-2026/nhan-dinh-panama-vs-croatia-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-colombia-vs-dr-congo-wc-2026/nhan-dinh-colombia-vs-dr-congo-wc-2026.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -944,9 +1043,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G72"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G90"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1348,7 +1447,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1362,7 +1461,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -1376,7 +1475,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>47</v>
       </c>
@@ -1390,7 +1489,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -1404,7 +1503,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -1418,7 +1517,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1432,7 +1531,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1446,7 +1545,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -1460,7 +1559,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -1474,7 +1573,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1488,7 +1587,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -1502,7 +1601,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1516,7 +1615,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>73</v>
       </c>
@@ -1530,7 +1629,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -1544,7 +1643,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>79</v>
       </c>
@@ -1558,7 +1657,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -1572,7 +1671,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>85</v>
       </c>
@@ -1586,7 +1685,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>88</v>
       </c>
@@ -1600,7 +1699,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -1614,7 +1713,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>94</v>
       </c>
@@ -1628,7 +1727,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="39" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>97</v>
       </c>
@@ -1642,7 +1741,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="40" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>100</v>
       </c>
@@ -1656,7 +1755,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>103</v>
       </c>
@@ -1670,7 +1769,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>106</v>
       </c>
@@ -1684,7 +1783,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>109</v>
       </c>
@@ -1698,7 +1797,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="44" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>112</v>
       </c>
@@ -1709,7 +1808,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>114</v>
       </c>
@@ -1720,7 +1819,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="46" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>116</v>
       </c>
@@ -1731,7 +1830,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>118</v>
       </c>
@@ -1742,7 +1841,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="48" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>120</v>
       </c>
@@ -1753,7 +1852,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>122</v>
       </c>
@@ -1767,7 +1866,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>125</v>
       </c>
@@ -1781,7 +1880,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>127</v>
       </c>
@@ -1795,7 +1894,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>129</v>
       </c>
@@ -1809,7 +1908,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>131</v>
       </c>
@@ -1823,7 +1922,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>133</v>
       </c>
@@ -1837,7 +1936,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>135</v>
       </c>
@@ -1851,7 +1950,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>137</v>
       </c>
@@ -1865,7 +1964,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>139</v>
       </c>
@@ -1879,7 +1978,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>142</v>
       </c>
@@ -1893,7 +1992,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="59" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -1907,7 +2006,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>148</v>
       </c>
@@ -1921,7 +2020,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>151</v>
       </c>
@@ -1935,7 +2034,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>154</v>
       </c>
@@ -1949,7 +2048,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>157</v>
       </c>
@@ -1963,7 +2062,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>159</v>
       </c>
@@ -1977,7 +2076,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="65" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>161</v>
       </c>
@@ -1991,7 +2090,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="66" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>164</v>
       </c>
@@ -2005,7 +2104,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="67" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>167</v>
       </c>
@@ -2019,7 +2118,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>170</v>
       </c>
@@ -2033,7 +2132,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>173</v>
       </c>
@@ -2047,7 +2146,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>176</v>
       </c>
@@ -2061,7 +2160,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>179</v>
       </c>
@@ -2075,7 +2174,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>181</v>
       </c>
@@ -2089,8 +2188,239 @@
         <v>182</v>
       </c>
     </row>
+    <row r="73" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>183</v>
+      </c>
+      <c r="D73" t="s">
+        <v>123</v>
+      </c>
+      <c r="E73" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>185</v>
+      </c>
+      <c r="E74" t="s">
+        <v>9</v>
+      </c>
+      <c r="F74" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>187</v>
+      </c>
+      <c r="E75" t="s">
+        <v>9</v>
+      </c>
+      <c r="F75" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>189</v>
+      </c>
+      <c r="E76" t="s">
+        <v>9</v>
+      </c>
+      <c r="F76" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>191</v>
+      </c>
+      <c r="E77" t="s">
+        <v>9</v>
+      </c>
+      <c r="F77" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>193</v>
+      </c>
+      <c r="E78" t="s">
+        <v>9</v>
+      </c>
+      <c r="F78" t="s">
+        <v>194</v>
+      </c>
+      <c r="G78" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>195</v>
+      </c>
+      <c r="D79" t="s">
+        <v>196</v>
+      </c>
+      <c r="E79" t="s">
+        <v>9</v>
+      </c>
+      <c r="F79" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>198</v>
+      </c>
+      <c r="D80" t="s">
+        <v>196</v>
+      </c>
+      <c r="E80" t="s">
+        <v>9</v>
+      </c>
+      <c r="F80" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>200</v>
+      </c>
+      <c r="D81" t="s">
+        <v>196</v>
+      </c>
+      <c r="E81" t="s">
+        <v>9</v>
+      </c>
+      <c r="F81" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>202</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="D82" t="s">
+        <v>203</v>
+      </c>
+      <c r="E82" t="s">
+        <v>9</v>
+      </c>
+      <c r="G82" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>205</v>
+      </c>
+      <c r="B83" t="s">
+        <v>9</v>
+      </c>
+      <c r="D83" t="s">
+        <v>203</v>
+      </c>
+      <c r="E83" t="s">
+        <v>9</v>
+      </c>
+      <c r="G83" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>206</v>
+      </c>
+      <c r="B84" t="s">
+        <v>9</v>
+      </c>
+      <c r="D84" t="s">
+        <v>203</v>
+      </c>
+      <c r="E84" t="s">
+        <v>9</v>
+      </c>
+      <c r="G84" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>207</v>
+      </c>
+      <c r="B85" t="s">
+        <v>9</v>
+      </c>
+      <c r="D85" t="s">
+        <v>203</v>
+      </c>
+      <c r="E85" t="s">
+        <v>9</v>
+      </c>
+      <c r="G85" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>208</v>
+      </c>
+      <c r="B86" t="s">
+        <v>9</v>
+      </c>
+      <c r="D86" t="s">
+        <v>203</v>
+      </c>
+      <c r="E86" t="s">
+        <v>9</v>
+      </c>
+      <c r="G86" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>209</v>
+      </c>
+      <c r="D87" t="s">
+        <v>196</v>
+      </c>
+      <c r="E87" t="s">
+        <v>9</v>
+      </c>
+      <c r="F87" t="s">
+        <v>210</v>
+      </c>
+      <c r="G87" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>213</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
content: add 5 WC2026 video inputs (recap/analysis/trivia batch)
- New inputs rendered via /video-queue (rows 86-90): na-uy-vs-senegal,
  dan-finisher-tuyen-anh, phap-vs-iraq, argentina-vs-ao, fact-1
- phap-vs-iraq: add dienbien (diễn biến) callout scene to script + plan
- Remove stale nhan-dinh-* input artifacts; update queue.xlsx statuses

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video/input/queue.xlsx
+++ b/video/input/queue.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79AD54A-B77C-4779-809A-1D211D253062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176"/>
   </bookViews>
   <sheets>
-    <sheet name="queue" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="queue" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="226">
   <si>
     <t>source</t>
   </si>
@@ -628,27 +622,6 @@
     <t>video/output/nhan-dinh-jordan-vs-algeria-wc-2026/video.mp4</t>
   </si>
   <si>
-    <t>video/input/cham-diem-bi-vs-iran-lukaku-mo-nhat/cham-diem-bi-vs-iran-lukaku-mo-nhat.txt</t>
-  </si>
-  <si>
-    <t>read-rewrite</t>
-  </si>
-  <si>
-    <t>Render failed</t>
-  </si>
-  <si>
-    <t>video/input/cham-diem-tay-ban-nha-vs-arab-saudi-oyarzabal/cham-diem-tay-ban-nha-vs-arab-saudi-oyarzabal.txt</t>
-  </si>
-  <si>
-    <t>video/input/owen-bao-ve-ronaldo-sau-tran-hoa-chdc-congo/owen-bao-ve-ronaldo-sau-tran-hoa-chdc-congo.txt</t>
-  </si>
-  <si>
-    <t>video/input/conceicao-bo-dao-nha-khong-co-nghia-vu-chuyen-cho-ronaldo/conceicao-bo-dao-nha-khong-co-nghia-vu-chuyen-cho-ronaldo.txt</t>
-  </si>
-  <si>
-    <t>video/input/top-10-cau-thu-vi-dai-nhat-lich-su-world-cup/top-10-cau-thu-vi-dai-nhat-lich-su-world-cup.txt</t>
-  </si>
-  <si>
     <t>video/input/nhan-dinh-bo-dao-nha-vs-uzbekistan-wc-2026/nhan-dinh-bo-dao-nha-vs-uzbekistan-wc-2026.txt</t>
   </si>
   <si>
@@ -658,23 +631,80 @@
     <t>video/input/nhan-dinh-anh-vs-ghana-wc-2026/nhan-dinh-anh-vs-ghana-wc-2026.txt</t>
   </si>
   <si>
+    <t>video/output/nhan-dinh-anh-vs-ghana-wc-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/nhan-dinh-panama-vs-croatia-wc-2026/nhan-dinh-panama-vs-croatia-wc-2026.txt</t>
   </si>
   <si>
+    <t>video/output/nhan-dinh-panama-vs-croatia-wc-2026/video.mp4</t>
+  </si>
+  <si>
     <t>video/input/nhan-dinh-colombia-vs-dr-congo-wc-2026/nhan-dinh-colombia-vs-dr-congo-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-colombia-vs-dr-congo-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-na-uy-vs-senegal-wc-2026/cham-diem-na-uy-vs-senegal-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite: Na Uy 3-2 Senegal (MATCH RECAP, 15 anh)</t>
+  </si>
+  <si>
+    <t>video/output/cham-diem-na-uy-vs-senegal-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/dan-finisher-tuyen-anh-wc-2026/dan-finisher-tuyen-anh-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite: dan finisher tuyen Anh (MATCH ANALYSIS, 7 anh)</t>
+  </si>
+  <si>
+    <t>video/output/dan-finisher-tuyen-anh-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-phap-vs-iraq-wc-2026/cham-diem-phap-vs-iraq-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite: Phap 3-0 Iraq (MATCH RECAP, 15 anh)</t>
+  </si>
+  <si>
+    <t>video/output/cham-diem-phap-vs-iraq-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/cham-diem-argentina-vs-ao-wc-2026/cham-diem-argentina-vs-ao-wc-2026.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite: Argentina 2-0 Ao, Messi ky luc (MATCH RECAP, 16 anh; Scaloni thay Paredes)</t>
+  </si>
+  <si>
+    <t>video/output/cham-diem-argentina-vs-ao-wc-2026/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/fact-1/fact-1.txt</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>refine + TRIVIA: 10 con so WC2026 (11 canh, 12 anh)</t>
+  </si>
+  <si>
+    <t>video/output/fact-1/video.mp4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -1043,9 +1073,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G90"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1447,7 +1477,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1461,7 +1491,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -1475,7 +1505,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>47</v>
       </c>
@@ -1489,7 +1519,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -1503,7 +1533,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -1517,7 +1547,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -1531,7 +1561,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>56</v>
       </c>
@@ -1545,7 +1575,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -1559,7 +1589,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -1573,7 +1603,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -1587,7 +1617,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>67</v>
       </c>
@@ -1601,7 +1631,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1615,7 +1645,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>73</v>
       </c>
@@ -1629,7 +1659,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -1643,7 +1673,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>79</v>
       </c>
@@ -1657,7 +1687,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>82</v>
       </c>
@@ -1671,7 +1701,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>85</v>
       </c>
@@ -1685,7 +1715,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>88</v>
       </c>
@@ -1699,7 +1729,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -1713,7 +1743,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>94</v>
       </c>
@@ -1727,7 +1757,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>97</v>
       </c>
@@ -1741,7 +1771,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>100</v>
       </c>
@@ -1755,7 +1785,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>103</v>
       </c>
@@ -1769,7 +1799,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>106</v>
       </c>
@@ -1783,7 +1813,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>109</v>
       </c>
@@ -1797,7 +1827,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>112</v>
       </c>
@@ -1808,7 +1838,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>114</v>
       </c>
@@ -1819,7 +1849,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>116</v>
       </c>
@@ -1830,7 +1860,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>118</v>
       </c>
@@ -1841,7 +1871,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>120</v>
       </c>
@@ -1852,7 +1882,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>122</v>
       </c>
@@ -1866,7 +1896,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>125</v>
       </c>
@@ -1880,7 +1910,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>127</v>
       </c>
@@ -1894,7 +1924,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>129</v>
       </c>
@@ -1908,7 +1938,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>131</v>
       </c>
@@ -1922,7 +1952,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>133</v>
       </c>
@@ -1936,7 +1966,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>135</v>
       </c>
@@ -1950,7 +1980,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>137</v>
       </c>
@@ -1964,7 +1994,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>139</v>
       </c>
@@ -1978,7 +2008,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>142</v>
       </c>
@@ -1992,7 +2022,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>145</v>
       </c>
@@ -2006,7 +2036,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>148</v>
       </c>
@@ -2020,7 +2050,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>151</v>
       </c>
@@ -2034,7 +2064,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>154</v>
       </c>
@@ -2048,7 +2078,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>157</v>
       </c>
@@ -2062,7 +2092,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>159</v>
       </c>
@@ -2076,7 +2106,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>161</v>
       </c>
@@ -2090,7 +2120,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>164</v>
       </c>
@@ -2104,7 +2134,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>167</v>
       </c>
@@ -2118,7 +2148,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>170</v>
       </c>
@@ -2132,7 +2162,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>173</v>
       </c>
@@ -2146,7 +2176,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>176</v>
       </c>
@@ -2160,7 +2190,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>179</v>
       </c>
@@ -2174,7 +2204,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>181</v>
       </c>
@@ -2188,7 +2218,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>183</v>
       </c>
@@ -2202,7 +2232,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>185</v>
       </c>
@@ -2213,7 +2243,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>187</v>
       </c>
@@ -2224,7 +2254,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>189</v>
       </c>
@@ -2235,7 +2265,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>191</v>
       </c>
@@ -2246,7 +2276,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="78" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" ht="14.4" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>193</v>
       </c>
@@ -2260,7 +2290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>195</v>
       </c>
@@ -2274,7 +2304,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>198</v>
       </c>
@@ -2288,7 +2318,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>200</v>
       </c>
@@ -2302,125 +2332,131 @@
         <v>201</v>
       </c>
     </row>
-    <row r="82" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" ht="14.4" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>202</v>
       </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
       <c r="D82" t="s">
+        <v>196</v>
+      </c>
+      <c r="E82" t="s">
+        <v>9</v>
+      </c>
+      <c r="F82" t="s">
         <v>203</v>
       </c>
-      <c r="E82" t="s">
-        <v>9</v>
-      </c>
       <c r="G82" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+      <c r="E83" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" t="s">
         <v>205</v>
       </c>
-      <c r="B83" t="s">
-        <v>9</v>
-      </c>
-      <c r="D83" t="s">
-        <v>203</v>
-      </c>
-      <c r="E83" t="s">
-        <v>9</v>
-      </c>
-      <c r="G83" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>206</v>
       </c>
-      <c r="B84" t="s">
-        <v>9</v>
-      </c>
-      <c r="D84" t="s">
-        <v>203</v>
-      </c>
       <c r="E84" t="s">
         <v>9</v>
       </c>
-      <c r="G84" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F84" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>207</v>
-      </c>
-      <c r="B85" t="s">
-        <v>9</v>
-      </c>
-      <c r="D85" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E85" t="s">
         <v>9</v>
       </c>
-      <c r="G85" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F85" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="86" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>208</v>
-      </c>
-      <c r="B86" t="s">
-        <v>9</v>
+        <v>210</v>
       </c>
       <c r="D86" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="E86" t="s">
         <v>9</v>
       </c>
-      <c r="G86" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F86" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="87" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D87" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
       <c r="E87" t="s">
         <v>9</v>
       </c>
       <c r="F87" t="s">
-        <v>210</v>
-      </c>
-      <c r="G87" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="88" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+        <v>216</v>
+      </c>
+      <c r="D88" t="s">
+        <v>217</v>
+      </c>
+      <c r="E88" t="s">
+        <v>9</v>
+      </c>
+      <c r="F88" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="89" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+        <v>219</v>
+      </c>
+      <c r="D89" t="s">
+        <v>220</v>
+      </c>
+      <c r="E89" t="s">
+        <v>9</v>
+      </c>
+      <c r="F89" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="90" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>213</v>
+        <v>222</v>
+      </c>
+      <c r="B90" t="s">
+        <v>223</v>
+      </c>
+      <c r="D90" t="s">
+        <v>224</v>
+      </c>
+      <c r="E90" t="s">
+        <v>9</v>
+      </c>
+      <c r="F90" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add new stories to podcast input: story155 to story161
- story155: Reflects on the struggles of a friend in entrepreneurship and the thin line between perseverance and stubbornness.
- story156: Discusses the challenges of adulthood and the importance of resilience during tough times.
- story157: A heartfelt tribute to Manchester United and the enduring love of a fan despite the team's struggles.
- story158: Explores the concepts of fate and debt in relationships, emphasizing the significance of connections.
- story159: Highlights Messi's journey and the silent struggles behind his success, contrasting it with Ronaldo's visible efforts.
- story160: Questions the feasibility of home ownership on a modest salary and encourages proactive financial planning.
- story161: Stresses the importance of self-love and personal growth in relationships, inspired by Matthew Hussey's insights.
</commit_message>
<xml_diff>
--- a/video/input/queue.xlsx
+++ b/video/input/queue.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="227">
   <si>
     <t>source</t>
   </si>
@@ -638,6 +638,63 @@
   </si>
   <si>
     <t>video/output/mu-ban-9-mua-2-carrick-doi-them/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/ke-thang-nguoi-thua-truoc-mua-ngoai-hang/ke-thang-nguoi-thua-truoc-mua-ngoai-hang.txt</t>
+  </si>
+  <si>
+    <t>video/output/ke-thang-nguoi-thua-truoc-mua-ngoai-hang/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/mourinho-toi-khong-can-rodri/mourinho-toi-khong-can-rodri.txt</t>
+  </si>
+  <si>
+    <t>video/output/mourinho-toi-khong-can-rodri/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/mu-hoi-mua-baleba-65-trieu-bang/mu-hoi-mua-baleba-65-trieu-bang.txt</t>
+  </si>
+  <si>
+    <t>read-rewrite (user paste)</t>
+  </si>
+  <si>
+    <t>video/output/mu-hoi-mua-baleba-65-trieu-bang/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-arsenal-vs-coventry/nhan-dinh-arsenal-vs-coventry.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-arsenal-vs-coventry/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-man-city-vs-bournemouth/nhan-dinh-man-city-vs-bournemouth.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-man-city-vs-bournemouth/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-fulham-vs-chelsea/nhan-dinh-fulham-vs-chelsea.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-fulham-vs-chelsea/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-hull-city-vs-man-united/nhan-dinh-hull-city-vs-man-united.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-hull-city-vs-man-united/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-newcastle-vs-liverpool/nhan-dinh-newcastle-vs-liverpool.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-newcastle-vs-liverpool/video.mp4</t>
+  </si>
+  <si>
+    <t>video/input/nhan-dinh-brentford-vs-tottenham/nhan-dinh-brentford-vs-tottenham.txt</t>
+  </si>
+  <si>
+    <t>video/output/nhan-dinh-brentford-vs-tottenham/video.mp4</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -2388,6 +2445,132 @@
         <v>207</v>
       </c>
     </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>208</v>
+      </c>
+      <c r="D97" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97" t="s">
+        <v>9</v>
+      </c>
+      <c r="F97" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>210</v>
+      </c>
+      <c r="D98" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98" t="s">
+        <v>9</v>
+      </c>
+      <c r="F98" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>212</v>
+      </c>
+      <c r="D99" t="s">
+        <v>213</v>
+      </c>
+      <c r="E99" t="s">
+        <v>9</v>
+      </c>
+      <c r="F99" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>215</v>
+      </c>
+      <c r="D100" t="s">
+        <v>14</v>
+      </c>
+      <c r="E100" t="s">
+        <v>9</v>
+      </c>
+      <c r="F100" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>217</v>
+      </c>
+      <c r="D101" t="s">
+        <v>14</v>
+      </c>
+      <c r="E101" t="s">
+        <v>9</v>
+      </c>
+      <c r="F101" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>219</v>
+      </c>
+      <c r="D102" t="s">
+        <v>14</v>
+      </c>
+      <c r="E102" t="s">
+        <v>9</v>
+      </c>
+      <c r="F102" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>221</v>
+      </c>
+      <c r="D103" t="s">
+        <v>14</v>
+      </c>
+      <c r="E103" t="s">
+        <v>9</v>
+      </c>
+      <c r="F103" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>223</v>
+      </c>
+      <c r="D104" t="s">
+        <v>14</v>
+      </c>
+      <c r="E104" t="s">
+        <v>9</v>
+      </c>
+      <c r="F104" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>225</v>
+      </c>
+      <c r="D105" t="s">
+        <v>14</v>
+      </c>
+      <c r="E105" t="s">
+        <v>9</v>
+      </c>
+      <c r="F105" t="s">
+        <v>226</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>